<commit_message>
Add screenshot display next to each step in Steps tab and update test case with Step 22
</commit_message>
<xml_diff>
--- a/test_case_table.xlsx
+++ b/test_case_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lollal/Documents/ai-agent-qa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EAB39FD-C163-1747-9BCF-F7349C4D76A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1584FE2A-7F49-314E-9CB3-6B1D0FB79CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="56">
   <si>
     <t>Step</t>
   </si>
@@ -173,19 +173,52 @@
   </si>
   <si>
     <t>//input[@data-testid="submission-name-input"]</t>
+  </si>
+  <si>
+    <t>//table[@data-testid="generic-table"]</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>verify</t>
+  </si>
+  <si>
+    <t>TABLE</t>
+  </si>
+  <si>
+    <t>Submission Name=spandana</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.9"/>
+      <color theme="1"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -208,8 +241,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="114.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.5" bestFit="1" customWidth="1"/>
@@ -1044,6 +1080,32 @@
       <c r="G24" t="s">
         <v>48</v>
       </c>
+      <c r="H24">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>